<commit_message>
Corregir inventario Ruge segun revision de Mariano (canas, platos, alargador, pala, cinta, Jefferson en Eventos)
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/INVENTARIO_2026_RUGE_actualizado_30ago2026.xlsx
+++ b/mariano-os/areas/ministerio/recursos/INVENTARIO_2026_RUGE_actualizado_30ago2026.xlsx
@@ -989,14 +989,14 @@
           <t>ADMINISTRACIÓN</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>GESTIONADO</t>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>GESTIONANDO</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Coordinado con contacto de Jonathan (via Marco Guanuchi), ~23-24€, retiro domingo.</t>
+          <t>Corregido 30 ago 2026 (Mariano): la nota de "ya coordinado, se retira el domingo" era incorrecta/de origen dudoso. Lo gestiona David y el todavia NO sabe con quien - falta contacto.</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Amazon 11,99€/rollo 5cmx10m, link B0BHQDDXJ7 - ⚠ el producto del link es amarilla fluorescente, no plateada, confirmar con Mariano si sirve igual.</t>
+          <t>⚠ A confirmar con Marco Jurado el 31 ago: el inventario oficial pone la comision de revision como solo "LOGISTICA" (sin "Y EVENTOS"), lo que por la regla ya confirmada significaria que es tarea de Logistica - pero Mariano recuerda que esto lo gestiona Eventos. Verificar cual es correcto antes de asignarlo. Amazon 11,99€/rollo, link B0BHQDDXJ7 - ademas el link es amarilla fluorescente, no plateada, confirmar si sirve igual.</t>
         </is>
       </c>
     </row>
@@ -1478,14 +1478,14 @@
           <t>ADMINISTRACIÓN</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>GESTIONADO</t>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>GESTIONANDO</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>David ya consiguio y grabo los platos que faltaban con "RUGE" (28 ago) - falta solo que envien la factura.</t>
+          <t>Corregido 30 ago 2026 (Mariano): Richard ya hizo los platos (segun David), pero no confirmo si los regala, los "siembra", o espera que se le pague - falta definir con Richard antes de dar esto por cerrado.</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>⚠ No se pudo cruzar con certeza contra "CARAMELO BLANCO" del listado de compra (unidad distinta, "bolsa 45 und") - confirmar con Marco Jurado si es el mismo item.</t>
+          <t>A confirmar con Marco Jurado el 31 ago (Mariano tampoco lo sabe con certeza): no se pudo cruzar contra "CARAMELO BLANCO" del listado de compra (unidad distinta, "bolsa 45 und").</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>A confirmar con Marcos Chiriguaya - reasignado de Julio a Eventos (comision de revision oficial).</t>
+          <t>Corregido 30 ago 2026: comision de revision oficial es Logistica y Eventos - Eventos gestiona. Encargado real de Eventos hoy es Jefferson (no Mauricio/Cristian). A confirmar con Marcos Chiriguaya el contacto.</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>Comision de revision oficial es Logistica y Eventos - segun la regla de Marco Jurado, Eventos (Mauricio/Cristian) gestiona/ejecuta, reasignado de Julio a Eventos.</t>
+          <t>Corregido 30 ago 2026: comision de revision oficial es Logistica y Eventos - Eventos gestiona. Encargado real de Eventos hoy es Jefferson (Mauricio y Cristian ya no estan en Eventos).</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2893,7 @@
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Comision de revision oficial es Logistica y Eventos - segun la regla de Marco Jurado, Eventos (Mauricio/Cristian) gestiona/ejecuta, reasignado de Julio a Eventos.</t>
+          <t>Corregido 30 ago 2026: comision de revision oficial es Logistica y Eventos - Eventos gestiona. Encargado real de Eventos hoy es Jefferson (Mauricio y Cristian ya no estan en Eventos).</t>
         </is>
       </c>
     </row>
@@ -4173,7 +4173,7 @@
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Marco Jurado ya le paso el contacto a Julio, que ya esta gestionando (28 ago).</t>
+          <t>Marco Jurado ya le paso el contacto a Julio, que ya esta gestionando (28 ago) - confirmar avance.</t>
         </is>
       </c>
     </row>
@@ -7011,14 +7011,14 @@
           <t>LOGISTÍCA</t>
         </is>
       </c>
-      <c r="H160" s="3" t="inlineStr">
-        <is>
-          <t>GESTIONADO</t>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>GESTIONANDO</t>
         </is>
       </c>
       <c r="I160" s="3" t="inlineStr">
         <is>
-          <t>Ya prestado por Iglesia Impact Valencia - solo falta probar que funcione (el amarillo grande puede estar roto).</t>
+          <t>Corregido 30 ago 2026 (Mariano): ninguno de los 2 alargadores de la iglesia sirve bien (uno no llega por largo, el otro es muy chico) - probablemente haya que comprar uno nuevo. Sin presupuesto todavia.</t>
         </is>
       </c>
     </row>
@@ -7448,9 +7448,9 @@
           <t>PENDIENTE GESTIONAR</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr">
-        <is>
-          <t>LOGÍSTICA</t>
+      <c r="G170" s="3" t="inlineStr">
+        <is>
+          <t>COCINA</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="I170" s="3" t="inlineStr">
         <is>
-          <t>⚠ Contradiccion sin resolver: el inventario oficial dice comision de revision COCINA, pero se asigno a Logistica en la llamada del 24 ago - confirmar con Marco Jurado. Compra via cuenta de Amazon especifica de Ruge (no la personal de Julio), pedir factura.</t>
+          <t>Corregido 30 ago 2026 (Mariano): si el inventario oficial dice Cocina, es Cocina - la llamada del 24 ago la habia asignado mal a Logistica. Avisar a Adrian Rivera (cocina). Compra via cuenta de Amazon especifica de Ruge, pedir factura.</t>
         </is>
       </c>
     </row>
@@ -10610,21 +10610,21 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Celdas en AZUL = modificadas por el sistema el 30 ago 2026 (columnas Estado actual / Checking)</t>
+          <t>Celdas en AZUL = modificadas por el sistema (columnas Gestion y finanzas / Estado actual / Checking)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Total de celdas modificadas: 35</t>
+          <t>Total de celdas modificadas: 33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Copialas a mano en el excel real de la nube, celda por celda, en la misma fila (buscando el nombre del artículo).</t>
+          <t>Version 30 ago 2026, corregida tras revision de Mariano (cañas, platos, alargador, pala metalica, cinta reflectante, Jefferson en Eventos).</t>
         </is>
       </c>
     </row>

</xml_diff>